<commit_message>
add bayesian; revise main text
</commit_message>
<xml_diff>
--- a/data/Site_information.xlsx
+++ b/data/Site_information.xlsx
@@ -1,26 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Quina_valleys\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985F41E1-31C0-4A0D-A36A-F3FA9F294E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54D7335-7FA9-4526-84AE-F234BE3CCAFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="89">
   <si>
     <t xml:space="preserve">name </t>
   </si>
@@ -200,9 +212,6 @@
   </si>
   <si>
     <t>SP</t>
-  </si>
-  <si>
-    <t>Heqing basin</t>
   </si>
   <si>
     <t>Dazhuang</t>
@@ -249,6 +258,66 @@
   </si>
   <si>
     <t xml:space="preserve">d_river_m </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Huangping basin</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Huajiaoqing</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>T4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>hilltop</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ganlanshudadi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Miaopotou</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Duimenshan</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dongyicun</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shiweigang</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pengjiadadi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Zhaokanzhuang</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dianweicun</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Xiaojianshan</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lujiacun</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>T3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -256,7 +325,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -295,6 +364,13 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -338,7 +414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -350,6 +426,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -630,6 +715,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="4">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{719FB610-9271-4949-8F52-0EC0C2472A0B}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;50677eba-79b2-4684-8261-8bf2650c43aa&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L28"/>
@@ -670,7 +777,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
@@ -685,7 +792,7 @@
         <v>9</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -708,7 +815,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H2" s="2">
         <v>1</v>
@@ -746,7 +853,7 @@
         <v>12</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H3" s="2">
         <v>0</v>
@@ -784,7 +891,7 @@
         <v>12</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H4" s="2">
         <v>1</v>
@@ -822,7 +929,7 @@
         <v>12</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H5" s="2">
         <v>1</v>
@@ -860,7 +967,7 @@
         <v>12</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H6" s="2">
         <v>1</v>
@@ -898,7 +1005,7 @@
         <v>12</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H7" s="2">
         <v>2</v>
@@ -936,7 +1043,7 @@
         <v>12</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H8" s="2">
         <v>2</v>
@@ -974,7 +1081,7 @@
         <v>12</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H9" s="2">
         <v>2</v>
@@ -1012,7 +1119,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H10" s="2">
         <v>10</v>
@@ -1050,7 +1157,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H11" s="2">
         <v>2</v>
@@ -1088,7 +1195,7 @@
         <v>12</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H12" s="2">
         <v>1</v>
@@ -1126,7 +1233,7 @@
         <v>12</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H13" s="2">
         <v>1</v>
@@ -1164,7 +1271,7 @@
         <v>12</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H14" s="2">
         <v>1</v>
@@ -1202,7 +1309,7 @@
         <v>12</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H15" s="2">
         <v>2</v>
@@ -1240,7 +1347,7 @@
         <v>12</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H16" s="2">
         <v>2</v>
@@ -1278,7 +1385,7 @@
         <v>12</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H17" s="2">
         <v>1</v>
@@ -1316,7 +1423,7 @@
         <v>12</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H18" s="2">
         <v>4</v>
@@ -1354,7 +1461,7 @@
         <v>12</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H19" s="2">
         <v>2</v>
@@ -1392,7 +1499,7 @@
         <v>12</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H20" s="2">
         <v>2</v>
@@ -1430,7 +1537,7 @@
         <v>12</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H21" s="2">
         <v>1</v>
@@ -1468,7 +1575,7 @@
         <v>12</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H22" s="2">
         <v>1</v>
@@ -1506,7 +1613,7 @@
         <v>12</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H23" s="2">
         <v>6</v>
@@ -1541,10 +1648,10 @@
         <v>1726</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H24" s="2">
         <v>19</v>
@@ -1564,10 +1671,10 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="C25" s="3">
         <v>26.004883</v>
@@ -1579,10 +1686,10 @@
         <v>1624</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H25" s="2">
         <v>6</v>
@@ -1594,7 +1701,7 @@
         <v>43</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L25" s="3">
         <v>339</v>
@@ -1602,10 +1709,10 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="C26" s="3">
         <v>26.036860999999998</v>
@@ -1617,10 +1724,10 @@
         <v>1805</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H26" s="2">
         <v>49</v>
@@ -1640,10 +1747,10 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="C27" s="3">
         <v>26.029722</v>
@@ -1655,10 +1762,10 @@
         <v>1540</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H27" s="2">
         <v>15</v>
@@ -1670,7 +1777,7 @@
         <v>40</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L27" s="3">
         <v>617</v>
@@ -1678,10 +1785,10 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="C28" s="3">
         <v>26.036722000000001</v>
@@ -1693,10 +1800,10 @@
         <v>1578</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H28" s="2">
         <v>31</v>
@@ -1708,11 +1815,347 @@
         <v>68</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L28" s="3">
         <v>917</v>
       </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD65DCCB-9181-496D-946D-52D078FCABAD}">
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17" style="2" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="10.88671875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="9" style="2"/>
+    <col min="5" max="5" width="14.44140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="10.21875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="5">
+        <v>25.989166999999998</v>
+      </c>
+      <c r="C2" s="5">
+        <v>100.532222</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1364</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" s="2">
+        <v>45</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="5">
+        <v>25.989722</v>
+      </c>
+      <c r="C3" s="5">
+        <v>100.531389</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1372</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" s="2">
+        <v>40</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="6">
+        <v>25.977499999999999</v>
+      </c>
+      <c r="C4" s="6">
+        <v>100.5425</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1374</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" s="2">
+        <v>31</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" s="6">
+        <v>25.911943999999998</v>
+      </c>
+      <c r="C5" s="6">
+        <v>100.46472199999999</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1674</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" s="2">
+        <v>41</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" s="6">
+        <v>25.908055999999998</v>
+      </c>
+      <c r="C6" s="6">
+        <v>100.465833</v>
+      </c>
+      <c r="D6" s="3">
+        <v>1687</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" s="3">
+        <v>60</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" s="6">
+        <v>25.902778000000001</v>
+      </c>
+      <c r="C7" s="6">
+        <v>100.47361100000001</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1666</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="3">
+        <v>51</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="6">
+        <v>25.878056000000001</v>
+      </c>
+      <c r="C8" s="6">
+        <v>100.469444</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1631</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="2">
+        <v>46</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="6">
+        <v>25.873611</v>
+      </c>
+      <c r="C9" s="6">
+        <v>100.47111099999999</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1621</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G9" s="3">
+        <v>45</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="6">
+        <v>25.867778000000001</v>
+      </c>
+      <c r="C10" s="6">
+        <v>100.477222</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1568</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G10" s="3">
+        <v>50</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="7">
+        <v>25.876389</v>
+      </c>
+      <c r="C11" s="6">
+        <v>100.492778</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1672</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11" s="2">
+        <v>130</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B12" s="7">
+        <v>25.865556000000002</v>
+      </c>
+      <c r="C12" s="6">
+        <v>100.498611</v>
+      </c>
+      <c r="D12" s="2">
+        <v>1634</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G12" s="2">
+        <v>69</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="J12"/>
+      <c r="K12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>